<commit_message>
Update Daily Adjustments template and parser to concise 4-column format: วันที่, รหัสพนักงาน, เครื่องจักรที่ไปทำ OT (OT Machine), เวลา
</commit_message>
<xml_diff>
--- a/Daily_Adjustments_Template.xlsx
+++ b/Daily_Adjustments_Template.xlsx
@@ -399,50 +399,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:D5"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="45.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>วันที่ (DD/MM/YYYY)</v>
+        <v>วันที่</v>
       </c>
       <c r="B1" t="str">
         <v>รหัสพนักงาน</v>
       </c>
       <c r="C1" t="str">
-        <v>ชื่อ - นามสกุล</v>
+        <v>เครื่องจักรที่ไปทำ OT (OT Machine)</v>
       </c>
       <c r="D1" t="str">
-        <v>แผนก/Cost Center</v>
-      </c>
-      <c r="E1" t="str">
-        <v>เครื่องประจำเดิม</v>
-      </c>
-      <c r="F1" t="str">
-        <v>1. ย้ายเครื่องกะปกติ</v>
-      </c>
-      <c r="G1" t="str">
-        <v>2. ย้ายเครื่องทำ OT</v>
-      </c>
-      <c r="H1" t="str">
-        <v>3. เวลาเข้าพิเศษ (HH:MM)</v>
-      </c>
-      <c r="I1" t="str">
-        <v>4. เวลาออกพิเศษ (HH:MM)</v>
-      </c>
-      <c r="J1" t="str">
-        <v>เหตุผล / หมายเหตุ</v>
+        <v>เวลา</v>
       </c>
     </row>
     <row r="2">
@@ -453,28 +429,10 @@
         <v>11848</v>
       </c>
       <c r="C2" t="str">
-        <v>วีระพันธ์ นุตะดี</v>
+        <v>320 BANBURY # 2</v>
       </c>
       <c r="D2" t="str">
-        <v>3200</v>
-      </c>
-      <c r="E2" t="str">
-        <v>320 BANBURY # 1</v>
-      </c>
-      <c r="F2" t="str">
         <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>320 BANBURY # 2</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v>ทำ OT กะ 3 ช่วย Mixer 2</v>
       </c>
     </row>
     <row r="3">
@@ -482,31 +440,13 @@
         <v>13/09/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12128</v>
+        <v>03027</v>
       </c>
       <c r="C3" t="str">
-        <v>พายุ บุญมาใส</v>
+        <v>320 BANBURY # 2</v>
       </c>
       <c r="D3" t="str">
-        <v>3200</v>
-      </c>
-      <c r="E3" t="str">
-        <v>320 BANBURY # 1</v>
-      </c>
-      <c r="F3" t="str">
-        <v>320 BANBURY # 2</v>
-      </c>
-      <c r="G3" t="str">
         <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v>ย้ายไปประจำ Mixer 2 กะ 1 แทนคนที่ลา</v>
       </c>
     </row>
     <row r="4">
@@ -517,28 +457,10 @@
         <v>12140</v>
       </c>
       <c r="C4" t="str">
-        <v>ถวิล ลืมอินทร์</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>3200</v>
-      </c>
-      <c r="E4" t="str">
-        <v>320 BANBURY # 1</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>11:00</v>
-      </c>
-      <c r="I4" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="J4" t="str">
-        <v>หัวหน้างานสั่งให้มาทำงานเวลาพิเศษ 11:00-19:00 (ไม่คิดสาย)</v>
+        <v>11:00 - 19:00</v>
       </c>
     </row>
     <row r="5">
@@ -546,36 +468,18 @@
         <v>13/09/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12412</v>
+        <v>12128</v>
       </c>
       <c r="C5" t="str">
-        <v>พิษณุ ช้างชน</v>
+        <v>320 BANBURY # 2</v>
       </c>
       <c r="D5" t="str">
-        <v>4300</v>
-      </c>
-      <c r="E5" t="str">
-        <v>430 Quad</v>
-      </c>
-      <c r="F5" t="str">
         <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>430 6"x8" Tuber</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v>ทำ OT กะ 3 ไปช่วยเครื่อง Tuber 6x8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -837,7 +741,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>หัวข้อ</v>
+        <v>คอลัมน์ (4 ช่อง)</v>
       </c>
       <c r="B1" t="str">
         <v>คำอธิบาย</v>
@@ -845,34 +749,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>รูปแบบที่ 1: กะตัวเอง ย้ายไปทำเครื่องอื่น (Normal Shift Transfer)</v>
+        <v>1. วันที่</v>
       </c>
       <c r="B2" t="str">
-        <v>กรอกชื่อเครื่องจักรเป้าหมายในช่อง "1. ย้ายเครื่องกะปกติ" -&gt; ระบบจะโอนยอดคนปกติ 1 คนไปนับที่เครื่องใหม่ทันที</v>
+        <v>วันที่ที่ต้องการปรับเปลี่ยน เช่น 13/09/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>รูปแบบที่ 2: กะตัวเองทำเครื่องเดิม และทำ OT เครื่องอื่น (OT Transfer)</v>
+        <v>2. รหัสพนักงาน</v>
       </c>
       <c r="B3" t="str">
-        <v>กรอกชื่อเครื่องจักรเป้าหมายในช่อง "2. ย้ายเครื่องทำ OT" -&gt; กำลังพลกะปกติจะอยู่เครื่องเดิม แต่ชั่วโมงและยอดกำลังพล OT จะโอนไปเติมให้เครื่องที่ไปช่วยทำ OT</v>
+        <v>รหัสพนักงาน 5 หลัก เช่น 11848</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>รูปแบบที่ 3: เวลาเข้า-ออกพิเศษตามที่หัวหน้างานสั่ง (Custom Shift Timing)</v>
+        <v>3. เครื่องจักรที่ไปทำ OT (OT Machine)</v>
       </c>
       <c r="B4" t="str">
-        <v>กรอกเวลาในช่อง "3. เวลาเข้าพิเศษ (HH:MM)" เช่น 11:00 -&gt; ระบบจะไม่คิดว่าสาย (isLate = false) และนับชั่วโมงทำงานปกติครบ 8 ชม.</v>
+        <v>ใส่ชื่อเครื่องจักรที่พนักงานไปทำ OT เช่น 320 BANBURY # 2 หรือ Mixer 2 (หากเป็นการย้ายกะปกติก็สามารถใส่เครื่องจักรที่ไปทำได้)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>คำแนะนำการระบุชื่อเครื่องจักร</v>
+        <v>4. เวลา</v>
       </c>
       <c r="B5" t="str">
-        <v>สามารถก๊อปปี้ชื่อเครื่องจักรจากแผ่นงาน "Standard_Machine_List" มาใส่ได้เลย หรือพิมพ์ชื่อย่อ เช่น Mixer 2, Quad, Tuber ระบบจะค้นหาให้อัตโนมัติ</v>
+        <v>กรณีหัวหน้าสั่งให้มาทำงานเวลาพิเศษ เช่น 11:00 หรือ 11:00 - 19:00 (ระบบจะไม่คิดสาย)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix daily adjustments syncing from T drive folder and robust date matching
</commit_message>
<xml_diff>
--- a/Daily_Adjustments_Template.xlsx
+++ b/Daily_Adjustments_Template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -698,7 +698,7 @@
         <v>16/09/2026</v>
       </c>
       <c r="B22">
-        <v>12626</v>
+        <v>12676</v>
       </c>
       <c r="C22" t="str">
         <v>Chaffer Lay-up</v>
@@ -715,15 +715,85 @@
         <v>12255</v>
       </c>
       <c r="C23" t="str">
-        <v>Trucker 4roll#1</v>
+        <v>แทน WAS</v>
       </c>
       <c r="D23" t="str">
         <v>23.00-07.00</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B24">
+        <v>12890</v>
+      </c>
+      <c r="C24" t="str">
+        <v xml:space="preserve">Pigment </v>
+      </c>
+      <c r="D24" t="str">
+        <v>23.00-07.00</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B25">
+        <v>10705</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Band 54</v>
+      </c>
+      <c r="D25" t="str">
+        <v>23.00-07.00</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B26">
+        <v>12809</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Chaffer Lay-up</v>
+      </c>
+      <c r="D26" t="str">
+        <v>07.00-15.00</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B27">
+        <v>12732</v>
+      </c>
+      <c r="C27" t="str">
+        <v xml:space="preserve">Pigment </v>
+      </c>
+      <c r="D27" t="str">
+        <v>23.00-07.00</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B28">
+        <v>12890</v>
+      </c>
+      <c r="C28" t="str">
+        <v xml:space="preserve">Pigment </v>
+      </c>
+      <c r="D28" t="str">
+        <v>23.00-07.00</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>